<commit_message>
fix: real DOM locators — p.zf-module-label drag source, customSelect_scheduleBy frequency, raw quoted text for verify steps
</commit_message>
<xml_diff>
--- a/manualtestcasedoc/Settings_standalone.xlsx
+++ b/manualtestcasedoc/Settings_standalone.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="100">
   <si>
     <t>S.No</t>
   </si>
@@ -288,13 +288,22 @@
     <t>Step13</t>
   </si>
   <si>
+    <t>Select any option in Connections field</t>
+  </si>
+  <si>
+    <t>We can able to choose any connections</t>
+  </si>
+  <si>
+    <t>Step14</t>
+  </si>
+  <si>
     <t>give input as test in message field</t>
   </si>
   <si>
     <t>Able to give input as mentioned</t>
   </si>
   <si>
-    <t>Step14</t>
+    <t>Step15</t>
   </si>
   <si>
     <t>Select 1st option in To Field</t>
@@ -303,10 +312,10 @@
     <t>Able to select option in To field</t>
   </si>
   <si>
-    <t>Step15</t>
+    <t>Step16</t>
   </si>
   <si>
-    <t>Step16</t>
+    <t>Step17</t>
   </si>
   <si>
     <t>Swith ON the flow</t>
@@ -314,12 +323,53 @@
   <si>
     <t>flow should not be SwitchedON</t>
   </si>
+  <si>
+    <t>CreateFlowSendMail</t>
+  </si>
+  <si>
+    <t>Create schedulerflow with SendMail action</t>
+  </si>
+  <si>
+    <t>Provide FlowName as "sendmailflow" in Flow Name field</t>
+  </si>
+  <si>
+    <t>Click Build-ins Subtab</t>
+  </si>
+  <si>
+    <t>Build-ins subtab should be clicked</t>
+  </si>
+  <si>
+    <t>Click Notification Section</t>
+  </si>
+  <si>
+    <t>Notification section should be expanded</t>
+  </si>
+  <si>
+    <t>Drag and Drop the "Send EMail" action into Trigger box</t>
+  </si>
+  <si>
+    <t>Send Mail action should be drag and dropped and SendMail popup should be opened</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Give input as </t>
+    </r>
+    <r>
+      <t>tmaniflow@gmail.com</t>
+    </r>
+    <r>
+      <t xml:space="preserve"> in "To" field</t>
+    </r>
+  </si>
+  <si>
+    <t>Give input as Automation in "Subject" field</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -349,6 +399,12 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0563C1"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -460,7 +516,7 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -530,6 +586,9 @@
     <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0">
+      <alignment vertical="bottom"/>
+    </xf>
     <xf borderId="5" fillId="4" fontId="3" numFmtId="3" xfId="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
     </xf>
@@ -555,7 +614,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main">
-  <dimension ref="A1:J497"/>
+  <dimension ref="A1:J498"/>
   <sheetFormatPr defaultRowHeight="14.0" customHeight="1"/>
   <cols>
     <col min="1" max="1" style="1" width="8.87"/>
@@ -1433,7 +1492,6 @@
       <c r="BI12" s="2"/>
       <c r="BJ12" s="2"/>
       <c r="BK12" s="2"/>
-      <c r="BZT12" s="2"/>
     </row>
     <row r="13" customHeight="1" ht="17.0" customFormat="1" s="2">
       <c r="A13" s="18"/>
@@ -1986,10 +2044,10 @@
         <v>82</v>
       </c>
       <c r="F25" s="22" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="G25" s="19" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="H25" s="14"/>
       <c r="I25" s="21"/>
@@ -2028,13 +2086,13 @@
         <v>14</v>
       </c>
       <c r="E26" s="19" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F26" s="22" t="s">
-        <v>84</v>
+        <v>65</v>
       </c>
       <c r="G26" s="19" t="s">
-        <v>85</v>
+        <v>66</v>
       </c>
       <c r="H26" s="14"/>
       <c r="I26" s="21"/>
@@ -2066,13 +2124,21 @@
       <c r="AI26" s="14"/>
     </row>
     <row r="27" customHeight="1" ht="17.0" customFormat="1" s="2">
-      <c r="A27" s="21"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
+      <c r="A27" s="18"/>
+      <c r="B27" s="19"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E27" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="F27" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="G27" s="19" t="s">
+        <v>88</v>
+      </c>
       <c r="H27" s="14"/>
       <c r="I27" s="21"/>
       <c r="J27" s="14"/>
@@ -2102,14 +2168,22 @@
       <c r="AH27" s="14"/>
       <c r="AI27" s="14"/>
     </row>
-    <row r="28" customHeight="1" ht="17.0" customFormat="1" s="2">
-      <c r="A28" s="21"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
+    <row r="28" customHeight="1" ht="45.0" customFormat="1" s="2">
+      <c r="A28" s="18">
+        <v>3.0</v>
+      </c>
+      <c r="B28" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="C28" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="D28" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" s="19"/>
+      <c r="F28" s="20"/>
+      <c r="G28" s="20"/>
       <c r="H28" s="14"/>
       <c r="I28" s="21"/>
       <c r="J28" s="14"/>
@@ -2140,13 +2214,21 @@
       <c r="AI28" s="14"/>
     </row>
     <row r="29" customHeight="1" ht="17.0" customFormat="1" s="2">
-      <c r="A29" s="21"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
+      <c r="A29" s="18"/>
+      <c r="B29" s="19"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E29" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="F29" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="G29" s="19" t="s">
+        <v>42</v>
+      </c>
       <c r="H29" s="14"/>
       <c r="I29" s="21"/>
       <c r="J29" s="14"/>
@@ -2177,13 +2259,21 @@
       <c r="AI29" s="14"/>
     </row>
     <row r="30" customHeight="1" ht="17.0" customFormat="1" s="2">
-      <c r="A30" s="21"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
+      <c r="A30" s="18"/>
+      <c r="B30" s="19"/>
+      <c r="C30" s="19"/>
+      <c r="D30" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E30" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="F30" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="G30" s="19" t="s">
+        <v>45</v>
+      </c>
       <c r="H30" s="14"/>
       <c r="I30" s="21"/>
       <c r="J30" s="14"/>
@@ -2214,13 +2304,21 @@
       <c r="AI30" s="14"/>
     </row>
     <row r="31" customHeight="1" ht="17.0" customFormat="1" s="2">
-      <c r="A31" s="21"/>
-      <c r="B31" s="14"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="14"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14"/>
-      <c r="G31" s="14"/>
+      <c r="A31" s="18"/>
+      <c r="B31" s="19"/>
+      <c r="C31" s="19"/>
+      <c r="D31" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E31" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="F31" s="22" t="s">
+        <v>91</v>
+      </c>
+      <c r="G31" s="19" t="s">
+        <v>48</v>
+      </c>
       <c r="H31" s="14"/>
       <c r="I31" s="21"/>
       <c r="J31" s="14"/>
@@ -2251,13 +2349,21 @@
       <c r="AI31" s="14"/>
     </row>
     <row r="32" customHeight="1" ht="17.0" customFormat="1" s="2">
-      <c r="A32" s="21"/>
-      <c r="B32" s="14"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="14"/>
-      <c r="E32" s="14"/>
-      <c r="F32" s="14"/>
-      <c r="G32" s="14"/>
+      <c r="A32" s="18"/>
+      <c r="B32" s="19"/>
+      <c r="C32" s="19"/>
+      <c r="D32" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E32" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="F32" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="G32" s="19" t="s">
+        <v>51</v>
+      </c>
       <c r="H32" s="14"/>
       <c r="I32" s="21"/>
       <c r="J32" s="14"/>
@@ -2288,13 +2394,21 @@
       <c r="AI32" s="14"/>
     </row>
     <row r="33" customHeight="1" ht="17.0" customFormat="1" s="2">
-      <c r="A33" s="21"/>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
+      <c r="A33" s="18"/>
+      <c r="B33" s="19"/>
+      <c r="C33" s="19"/>
+      <c r="D33" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E33" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="F33" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="G33" s="19" t="s">
+        <v>54</v>
+      </c>
       <c r="H33" s="14"/>
       <c r="I33" s="21"/>
       <c r="J33" s="14"/>
@@ -2325,13 +2439,21 @@
       <c r="AI33" s="14"/>
     </row>
     <row r="34" customHeight="1" ht="17.0" customFormat="1" s="2">
-      <c r="A34" s="21"/>
-      <c r="B34" s="14"/>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="14"/>
+      <c r="A34" s="18"/>
+      <c r="B34" s="19"/>
+      <c r="C34" s="19"/>
+      <c r="D34" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E34" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="F34" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="G34" s="19" t="s">
+        <v>57</v>
+      </c>
       <c r="H34" s="14"/>
       <c r="I34" s="21"/>
       <c r="J34" s="14"/>
@@ -2362,13 +2484,21 @@
       <c r="AI34" s="14"/>
     </row>
     <row r="35" customHeight="1" ht="17.0" customFormat="1" s="2">
-      <c r="A35" s="21"/>
-      <c r="B35" s="14"/>
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14"/>
+      <c r="A35" s="18"/>
+      <c r="B35" s="19"/>
+      <c r="C35" s="19"/>
+      <c r="D35" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E35" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="F35" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="G35" s="19" t="s">
+        <v>60</v>
+      </c>
       <c r="H35" s="14"/>
       <c r="I35" s="21"/>
       <c r="J35" s="14"/>
@@ -2399,13 +2529,21 @@
       <c r="AI35" s="14"/>
     </row>
     <row r="36" customHeight="1" ht="17.0" customFormat="1" s="2">
-      <c r="A36" s="21"/>
-      <c r="B36" s="14"/>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="14"/>
-      <c r="G36" s="14"/>
+      <c r="A36" s="18"/>
+      <c r="B36" s="19"/>
+      <c r="C36" s="19"/>
+      <c r="D36" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E36" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="F36" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="G36" s="19" t="s">
+        <v>63</v>
+      </c>
       <c r="H36" s="14"/>
       <c r="I36" s="21"/>
       <c r="J36" s="14"/>
@@ -2436,13 +2574,21 @@
       <c r="AI36" s="14"/>
     </row>
     <row r="37" customHeight="1" ht="17.0" customFormat="1" s="2">
-      <c r="A37" s="21"/>
-      <c r="B37" s="14"/>
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
-      <c r="G37" s="14"/>
+      <c r="A37" s="18"/>
+      <c r="B37" s="19"/>
+      <c r="C37" s="19"/>
+      <c r="D37" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E37" s="19" t="s">
+        <v>64</v>
+      </c>
+      <c r="F37" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="G37" s="19" t="s">
+        <v>66</v>
+      </c>
       <c r="H37" s="14"/>
       <c r="I37" s="21"/>
       <c r="J37" s="14"/>
@@ -2473,13 +2619,21 @@
       <c r="AI37" s="14"/>
     </row>
     <row r="38" customHeight="1" ht="17.0" customFormat="1" s="2">
-      <c r="A38" s="21"/>
-      <c r="B38" s="14"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
-      <c r="F38" s="14"/>
-      <c r="G38" s="14"/>
+      <c r="A38" s="18"/>
+      <c r="B38" s="19"/>
+      <c r="C38" s="19"/>
+      <c r="D38" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E38" s="19" t="s">
+        <v>67</v>
+      </c>
+      <c r="F38" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="G38" s="19" t="s">
+        <v>93</v>
+      </c>
       <c r="H38" s="14"/>
       <c r="I38" s="21"/>
       <c r="J38" s="14"/>
@@ -2510,13 +2664,21 @@
       <c r="AI38" s="14"/>
     </row>
     <row r="39" customHeight="1" ht="17.0" customFormat="1" s="2">
-      <c r="A39" s="21"/>
-      <c r="B39" s="14"/>
-      <c r="C39" s="14"/>
-      <c r="D39" s="14"/>
-      <c r="E39" s="14"/>
-      <c r="F39" s="14"/>
-      <c r="G39" s="14"/>
+      <c r="A39" s="18"/>
+      <c r="B39" s="19"/>
+      <c r="C39" s="19"/>
+      <c r="D39" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E39" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="F39" s="22" t="s">
+        <v>94</v>
+      </c>
+      <c r="G39" s="19" t="s">
+        <v>95</v>
+      </c>
       <c r="H39" s="14"/>
       <c r="I39" s="21"/>
       <c r="J39" s="14"/>
@@ -2547,13 +2709,21 @@
       <c r="AI39" s="14"/>
     </row>
     <row r="40" customHeight="1" ht="17.0" customFormat="1" s="2">
-      <c r="A40" s="21"/>
-      <c r="B40" s="14"/>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="14"/>
-      <c r="G40" s="14"/>
+      <c r="A40" s="18"/>
+      <c r="B40" s="19"/>
+      <c r="C40" s="19"/>
+      <c r="D40" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E40" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="F40" s="22" t="s">
+        <v>96</v>
+      </c>
+      <c r="G40" s="19" t="s">
+        <v>97</v>
+      </c>
       <c r="H40" s="14"/>
       <c r="I40" s="21"/>
       <c r="J40" s="14"/>
@@ -2584,13 +2754,21 @@
       <c r="AI40" s="14"/>
     </row>
     <row r="41" customHeight="1" ht="17.0" customFormat="1" s="2">
-      <c r="A41" s="21"/>
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="14"/>
-      <c r="F41" s="14"/>
-      <c r="G41" s="14"/>
+      <c r="A41" s="18"/>
+      <c r="B41" s="19"/>
+      <c r="C41" s="19"/>
+      <c r="D41" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E41" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="F41" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="G41" s="19" t="s">
+        <v>81</v>
+      </c>
       <c r="H41" s="14"/>
       <c r="I41" s="21"/>
       <c r="J41" s="14"/>
@@ -2621,13 +2799,21 @@
       <c r="AI41" s="14"/>
     </row>
     <row r="42" customHeight="1" ht="17.0" customFormat="1" s="2">
-      <c r="A42" s="21"/>
-      <c r="B42" s="14"/>
-      <c r="C42" s="14"/>
-      <c r="D42" s="14"/>
-      <c r="E42" s="14"/>
-      <c r="F42" s="14"/>
-      <c r="G42" s="14"/>
+      <c r="A42" s="18"/>
+      <c r="B42" s="19"/>
+      <c r="C42" s="19"/>
+      <c r="D42" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E42" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="F42" s="22" t="s">
+        <v>99</v>
+      </c>
+      <c r="G42" s="19" t="s">
+        <v>81</v>
+      </c>
       <c r="H42" s="14"/>
       <c r="I42" s="21"/>
       <c r="J42" s="14"/>
@@ -2658,13 +2844,21 @@
       <c r="AI42" s="14"/>
     </row>
     <row r="43" customHeight="1" ht="17.0" customFormat="1" s="2">
-      <c r="A43" s="21"/>
-      <c r="B43" s="14"/>
-      <c r="C43" s="14"/>
-      <c r="D43" s="14"/>
-      <c r="E43" s="14"/>
-      <c r="F43" s="14"/>
-      <c r="G43" s="14"/>
+      <c r="A43" s="18"/>
+      <c r="B43" s="19"/>
+      <c r="C43" s="19"/>
+      <c r="D43" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E43" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="F43" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="G43" s="19" t="s">
+        <v>66</v>
+      </c>
       <c r="H43" s="14"/>
       <c r="I43" s="21"/>
       <c r="J43" s="14"/>
@@ -2695,13 +2889,21 @@
       <c r="AI43" s="14"/>
     </row>
     <row r="44" customHeight="1" ht="17.0" customFormat="1" s="2">
-      <c r="A44" s="21"/>
-      <c r="B44" s="14"/>
-      <c r="C44" s="14"/>
-      <c r="D44" s="14"/>
-      <c r="E44" s="14"/>
-      <c r="F44" s="14"/>
-      <c r="G44" s="14"/>
+      <c r="A44" s="18"/>
+      <c r="B44" s="19"/>
+      <c r="C44" s="19"/>
+      <c r="D44" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E44" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="F44" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="G44" s="19" t="s">
+        <v>88</v>
+      </c>
       <c r="H44" s="14"/>
       <c r="I44" s="21"/>
       <c r="J44" s="14"/>
@@ -19455,78 +19657,118 @@
       <c r="AH496" s="14"/>
       <c r="AI496" s="14"/>
     </row>
-    <row r="497" customHeight="1" ht="17.0" customFormat="1" s="1">
-      <c r="A497" s="23">
-        <f>COUNTA(A2:A496)</f>
-        <v>2.0</v>
+    <row r="497" customHeight="1" ht="17.0" customFormat="1" s="2">
+      <c r="A497" s="21"/>
+      <c r="B497" s="14"/>
+      <c r="C497" s="14"/>
+      <c r="D497" s="14"/>
+      <c r="E497" s="14"/>
+      <c r="F497" s="14"/>
+      <c r="G497" s="14"/>
+      <c r="H497" s="14"/>
+      <c r="I497" s="21"/>
+      <c r="J497" s="14"/>
+      <c r="K497" s="14"/>
+      <c r="L497" s="14"/>
+      <c r="M497" s="14"/>
+      <c r="N497" s="14"/>
+      <c r="O497" s="14"/>
+      <c r="P497" s="14"/>
+      <c r="Q497" s="14"/>
+      <c r="R497" s="14"/>
+      <c r="S497" s="14"/>
+      <c r="T497" s="14"/>
+      <c r="U497" s="14"/>
+      <c r="V497" s="14"/>
+      <c r="W497" s="14"/>
+      <c r="X497" s="14"/>
+      <c r="Y497" s="14"/>
+      <c r="Z497" s="14"/>
+      <c r="AA497" s="14"/>
+      <c r="AB497" s="14"/>
+      <c r="AC497" s="14"/>
+      <c r="AD497" s="14"/>
+      <c r="AE497" s="14"/>
+      <c r="AF497" s="14"/>
+      <c r="AG497" s="14"/>
+      <c r="AH497" s="14"/>
+      <c r="AI497" s="14"/>
+    </row>
+    <row r="498" customHeight="1" ht="17.0" customFormat="1" s="1">
+      <c r="A498" s="24">
+        <f>COUNTA(A2:A497)</f>
+        <v>3.0</v>
       </c>
-      <c r="B497" s="24"/>
-      <c r="C497" s="24"/>
-      <c r="D497" s="24"/>
-      <c r="E497" s="24"/>
-      <c r="F497" s="24"/>
-      <c r="G497" s="24"/>
-      <c r="H497" s="24"/>
-      <c r="I497" s="23">
-        <f>COUNTA(I2:I496)</f>
+      <c r="B498" s="25"/>
+      <c r="C498" s="25"/>
+      <c r="D498" s="25"/>
+      <c r="E498" s="25"/>
+      <c r="F498" s="25"/>
+      <c r="G498" s="25"/>
+      <c r="H498" s="25"/>
+      <c r="I498" s="24">
+        <f>COUNTA(I2:I497)</f>
         <v>1.0</v>
       </c>
-      <c r="J497" s="24"/>
-      <c r="K497" s="24"/>
-      <c r="L497" s="24"/>
-      <c r="M497" s="24"/>
-      <c r="N497" s="24"/>
-      <c r="O497" s="24"/>
-      <c r="P497" s="24"/>
-      <c r="Q497" s="24"/>
-      <c r="R497" s="24"/>
-      <c r="S497" s="24"/>
-      <c r="T497" s="24"/>
-      <c r="U497" s="24"/>
-      <c r="V497" s="24"/>
-      <c r="W497" s="24"/>
-      <c r="X497" s="24"/>
-      <c r="Y497" s="24"/>
-      <c r="Z497" s="24"/>
-      <c r="AA497" s="24"/>
-      <c r="AB497" s="24"/>
-      <c r="AC497" s="24"/>
-      <c r="AD497" s="24"/>
-      <c r="AE497" s="24"/>
-      <c r="AF497" s="24"/>
-      <c r="AG497" s="24"/>
-      <c r="AH497" s="24"/>
-      <c r="AI497" s="24"/>
-      <c r="AJ497" s="15"/>
-      <c r="AK497" s="15"/>
-      <c r="AL497" s="2"/>
-      <c r="AM497" s="2"/>
-      <c r="AN497" s="2"/>
-      <c r="AO497" s="2"/>
-      <c r="AP497" s="2"/>
-      <c r="AQ497" s="2"/>
-      <c r="AR497" s="2"/>
-      <c r="AS497" s="2"/>
-      <c r="AT497" s="2"/>
-      <c r="AU497" s="2"/>
-      <c r="AV497" s="2"/>
-      <c r="AW497" s="2"/>
-      <c r="AX497" s="2"/>
-      <c r="AY497" s="2"/>
-      <c r="AZ497" s="2"/>
-      <c r="BA497" s="2"/>
-      <c r="BB497" s="2"/>
-      <c r="BC497" s="2"/>
-      <c r="BD497" s="2"/>
-      <c r="BE497" s="2"/>
-      <c r="BF497" s="2"/>
-      <c r="BG497" s="2"/>
-      <c r="BH497" s="2"/>
-      <c r="BI497" s="2"/>
-      <c r="BJ497" s="2"/>
-      <c r="BK497" s="2"/>
+      <c r="J498" s="25"/>
+      <c r="K498" s="25"/>
+      <c r="L498" s="25"/>
+      <c r="M498" s="25"/>
+      <c r="N498" s="25"/>
+      <c r="O498" s="25"/>
+      <c r="P498" s="25"/>
+      <c r="Q498" s="25"/>
+      <c r="R498" s="25"/>
+      <c r="S498" s="25"/>
+      <c r="T498" s="25"/>
+      <c r="U498" s="25"/>
+      <c r="V498" s="25"/>
+      <c r="W498" s="25"/>
+      <c r="X498" s="25"/>
+      <c r="Y498" s="25"/>
+      <c r="Z498" s="25"/>
+      <c r="AA498" s="25"/>
+      <c r="AB498" s="25"/>
+      <c r="AC498" s="25"/>
+      <c r="AD498" s="25"/>
+      <c r="AE498" s="25"/>
+      <c r="AF498" s="25"/>
+      <c r="AG498" s="25"/>
+      <c r="AH498" s="25"/>
+      <c r="AI498" s="25"/>
+      <c r="AJ498" s="15"/>
+      <c r="AK498" s="15"/>
+      <c r="AL498" s="2"/>
+      <c r="AM498" s="2"/>
+      <c r="AN498" s="2"/>
+      <c r="AO498" s="2"/>
+      <c r="AP498" s="2"/>
+      <c r="AQ498" s="2"/>
+      <c r="AR498" s="2"/>
+      <c r="AS498" s="2"/>
+      <c r="AT498" s="2"/>
+      <c r="AU498" s="2"/>
+      <c r="AV498" s="2"/>
+      <c r="AW498" s="2"/>
+      <c r="AX498" s="2"/>
+      <c r="AY498" s="2"/>
+      <c r="AZ498" s="2"/>
+      <c r="BA498" s="2"/>
+      <c r="BB498" s="2"/>
+      <c r="BC498" s="2"/>
+      <c r="BD498" s="2"/>
+      <c r="BE498" s="2"/>
+      <c r="BF498" s="2"/>
+      <c r="BG498" s="2"/>
+      <c r="BH498" s="2"/>
+      <c r="BI498" s="2"/>
+      <c r="BJ498" s="2"/>
+      <c r="BK498" s="2"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F41" r:id="rId1"/>
+  </hyperlinks>
   <extLst/>
 </worksheet>
 </file>
</xml_diff>